<commit_message>
Added Temperature Analysis due to it being an important criteria for Self Organizing Maps in our case
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/MPDI_Xianshuihe.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/MPDI_Xianshuihe.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\Gesammelte_Datenbanken\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/94a36cc37384f3e2/SPEICHER/Hochschule/7. Semester/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{141DDCD0-33E4-4661-B51D-90FE6CA76C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{141DDCD0-33E4-4661-B51D-90FE6CA76C8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0F7BD04-15B8-4AF5-B169-9B491E7F1DD9}"/>
   <bookViews>
-    <workbookView xWindow="1305" yWindow="4020" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$V$1:$V$281</definedName>
+  </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
@@ -688,6 +691,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:Y281"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -768,7 +772,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -836,7 +840,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -907,7 +911,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -975,7 +979,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -1043,7 +1047,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -1111,7 +1115,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>28</v>
       </c>
@@ -1173,7 +1177,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>29</v>
       </c>
@@ -1241,7 +1245,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>29</v>
       </c>
@@ -1309,7 +1313,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -1377,7 +1381,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -1445,7 +1449,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>30</v>
       </c>
@@ -1513,7 +1517,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -1581,7 +1585,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>31</v>
       </c>
@@ -1649,7 +1653,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>31</v>
       </c>
@@ -1717,7 +1721,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:25" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>31</v>
       </c>
@@ -1785,7 +1789,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>31</v>
       </c>
@@ -1850,7 +1854,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -1918,7 +1922,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>31</v>
       </c>
@@ -1986,7 +1990,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>32</v>
       </c>
@@ -2054,7 +2058,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>32</v>
       </c>
@@ -2122,7 +2126,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -2190,7 +2194,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -2258,7 +2262,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>33</v>
       </c>
@@ -2326,7 +2330,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>33</v>
       </c>
@@ -2394,7 +2398,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>34</v>
       </c>
@@ -2462,7 +2466,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>34</v>
       </c>
@@ -2530,7 +2534,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>34</v>
       </c>
@@ -2598,7 +2602,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>35</v>
       </c>
@@ -2666,7 +2670,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>36</v>
       </c>
@@ -2734,7 +2738,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -2802,7 +2806,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>36</v>
       </c>
@@ -2870,7 +2874,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>37</v>
       </c>
@@ -2938,7 +2942,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>37</v>
       </c>
@@ -3006,7 +3010,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>37</v>
       </c>
@@ -3074,7 +3078,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>37</v>
       </c>
@@ -3142,7 +3146,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>37</v>
       </c>
@@ -3210,7 +3214,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>38</v>
       </c>
@@ -3278,7 +3282,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -3346,7 +3350,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -3414,7 +3418,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -3482,7 +3486,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>40</v>
       </c>
@@ -3550,7 +3554,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>40</v>
       </c>
@@ -3618,7 +3622,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>41</v>
       </c>
@@ -3686,7 +3690,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>41</v>
       </c>
@@ -3754,7 +3758,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>41</v>
       </c>
@@ -3822,7 +3826,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>41</v>
       </c>
@@ -3890,7 +3894,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>41</v>
       </c>
@@ -3958,7 +3962,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>41</v>
       </c>
@@ -4026,7 +4030,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>42</v>
       </c>
@@ -4094,7 +4098,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>42</v>
       </c>
@@ -4162,7 +4166,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>42</v>
       </c>
@@ -4230,7 +4234,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>42</v>
       </c>
@@ -4298,7 +4302,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>42</v>
       </c>
@@ -4366,7 +4370,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>42</v>
       </c>
@@ -4434,7 +4438,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>42</v>
       </c>
@@ -4502,7 +4506,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>42</v>
       </c>
@@ -4570,7 +4574,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>42</v>
       </c>
@@ -4638,7 +4642,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>42</v>
       </c>
@@ -4706,7 +4710,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>42</v>
       </c>
@@ -4774,7 +4778,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>43</v>
       </c>
@@ -4842,7 +4846,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>43</v>
       </c>
@@ -4910,7 +4914,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>43</v>
       </c>
@@ -4978,7 +4982,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>43</v>
       </c>
@@ -5046,7 +5050,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>43</v>
       </c>
@@ -5114,7 +5118,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>43</v>
       </c>
@@ -5182,7 +5186,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>43</v>
       </c>
@@ -5250,7 +5254,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>43</v>
       </c>
@@ -5318,7 +5322,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>43</v>
       </c>
@@ -5386,7 +5390,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>43</v>
       </c>
@@ -5454,7 +5458,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>43</v>
       </c>
@@ -5522,7 +5526,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>44</v>
       </c>
@@ -5590,7 +5594,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>44</v>
       </c>
@@ -5658,7 +5662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>44</v>
       </c>
@@ -5726,7 +5730,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>44</v>
       </c>
@@ -5794,7 +5798,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>44</v>
       </c>
@@ -5862,7 +5866,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>45</v>
       </c>
@@ -5930,7 +5934,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>46</v>
       </c>
@@ -5998,7 +6002,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>46</v>
       </c>
@@ -6066,7 +6070,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>46</v>
       </c>
@@ -6134,7 +6138,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>47</v>
       </c>
@@ -6202,7 +6206,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>47</v>
       </c>
@@ -6270,7 +6274,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>47</v>
       </c>
@@ -6338,7 +6342,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>47</v>
       </c>
@@ -6406,7 +6410,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>47</v>
       </c>
@@ -6474,7 +6478,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>47</v>
       </c>
@@ -6542,7 +6546,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>47</v>
       </c>
@@ -6610,7 +6614,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>47</v>
       </c>
@@ -6678,7 +6682,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>47</v>
       </c>
@@ -6746,7 +6750,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>47</v>
       </c>
@@ -6814,7 +6818,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>47</v>
       </c>
@@ -6882,7 +6886,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>47</v>
       </c>
@@ -6950,7 +6954,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>48</v>
       </c>
@@ -7018,7 +7022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>48</v>
       </c>
@@ -7086,7 +7090,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>48</v>
       </c>
@@ -7154,7 +7158,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>48</v>
       </c>
@@ -7222,7 +7226,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>48</v>
       </c>
@@ -7290,7 +7294,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="98" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>48</v>
       </c>
@@ -7358,7 +7362,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>49</v>
       </c>
@@ -7426,7 +7430,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>49</v>
       </c>
@@ -7494,7 +7498,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>49</v>
       </c>
@@ -7562,7 +7566,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>49</v>
       </c>
@@ -7630,7 +7634,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>50</v>
       </c>
@@ -7698,7 +7702,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>50</v>
       </c>
@@ -7766,7 +7770,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>50</v>
       </c>
@@ -7834,7 +7838,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="106" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>50</v>
       </c>
@@ -7902,7 +7906,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="107" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>50</v>
       </c>
@@ -7970,7 +7974,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="108" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>50</v>
       </c>
@@ -8038,7 +8042,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="109" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>50</v>
       </c>
@@ -8106,7 +8110,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>50</v>
       </c>
@@ -8171,7 +8175,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="111" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>50</v>
       </c>
@@ -8236,7 +8240,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="112" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>50</v>
       </c>
@@ -8304,7 +8308,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="113" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>50</v>
       </c>
@@ -8372,7 +8376,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="114" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>50</v>
       </c>
@@ -8440,7 +8444,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="115" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>50</v>
       </c>
@@ -8508,7 +8512,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>50</v>
       </c>
@@ -8576,7 +8580,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="117" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>50</v>
       </c>
@@ -8644,7 +8648,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="118" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>50</v>
       </c>
@@ -8712,7 +8716,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="119" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>51</v>
       </c>
@@ -8780,7 +8784,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="120" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>51</v>
       </c>
@@ -8848,7 +8852,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>51</v>
       </c>
@@ -8916,7 +8920,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="122" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>51</v>
       </c>
@@ -8984,7 +8988,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="123" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>51</v>
       </c>
@@ -9052,7 +9056,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>51</v>
       </c>
@@ -9120,7 +9124,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="125" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>51</v>
       </c>
@@ -9188,7 +9192,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="126" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>52</v>
       </c>
@@ -9256,7 +9260,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="127" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>52</v>
       </c>
@@ -9324,7 +9328,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="128" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>52</v>
       </c>
@@ -9392,7 +9396,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="129" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>52</v>
       </c>
@@ -9460,7 +9464,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="130" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>52</v>
       </c>
@@ -9528,7 +9532,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="131" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>52</v>
       </c>
@@ -9596,7 +9600,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="132" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>52</v>
       </c>
@@ -9664,7 +9668,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="133" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>53</v>
       </c>
@@ -9732,7 +9736,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="134" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>53</v>
       </c>
@@ -9800,7 +9804,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="135" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>53</v>
       </c>
@@ -9868,7 +9872,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="136" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>53</v>
       </c>
@@ -9936,7 +9940,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="137" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>54</v>
       </c>
@@ -10004,7 +10008,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="138" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>54</v>
       </c>
@@ -10072,7 +10076,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="139" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>54</v>
       </c>
@@ -10140,7 +10144,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="140" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>54</v>
       </c>
@@ -10208,7 +10212,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="141" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>54</v>
       </c>
@@ -10276,7 +10280,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="142" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>54</v>
       </c>
@@ -10344,7 +10348,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="143" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>55</v>
       </c>
@@ -10412,7 +10416,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="144" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>55</v>
       </c>
@@ -10480,7 +10484,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="145" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>55</v>
       </c>
@@ -10548,7 +10552,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="146" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>55</v>
       </c>
@@ -10616,7 +10620,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="147" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>55</v>
       </c>
@@ -10684,7 +10688,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="148" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>55</v>
       </c>
@@ -10752,7 +10756,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="149" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>55</v>
       </c>
@@ -10820,7 +10824,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="150" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>55</v>
       </c>
@@ -10888,7 +10892,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="151" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>55</v>
       </c>
@@ -10956,7 +10960,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="152" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>55</v>
       </c>
@@ -11024,7 +11028,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="153" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>55</v>
       </c>
@@ -11092,7 +11096,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="154" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>55</v>
       </c>
@@ -11160,7 +11164,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="155" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>55</v>
       </c>
@@ -11228,7 +11232,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="156" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>55</v>
       </c>
@@ -11296,7 +11300,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="157" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>55</v>
       </c>
@@ -11364,7 +11368,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="158" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>55</v>
       </c>
@@ -11432,7 +11436,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="159" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>55</v>
       </c>
@@ -11500,7 +11504,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="160" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>56</v>
       </c>
@@ -11568,7 +11572,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="161" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>56</v>
       </c>
@@ -11636,7 +11640,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="162" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>56</v>
       </c>
@@ -11704,7 +11708,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="163" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>56</v>
       </c>
@@ -11772,7 +11776,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="164" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>56</v>
       </c>
@@ -11840,7 +11844,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="165" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>56</v>
       </c>
@@ -11908,7 +11912,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="166" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>56</v>
       </c>
@@ -11976,7 +11980,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="167" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>56</v>
       </c>
@@ -12044,7 +12048,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="168" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>56</v>
       </c>
@@ -12112,7 +12116,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="169" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>56</v>
       </c>
@@ -12180,7 +12184,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="170" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>56</v>
       </c>
@@ -12248,7 +12252,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="171" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>56</v>
       </c>
@@ -12316,7 +12320,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="172" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>56</v>
       </c>
@@ -12384,7 +12388,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="173" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>56</v>
       </c>
@@ -12452,7 +12456,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="174" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>56</v>
       </c>
@@ -12520,7 +12524,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="175" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>56</v>
       </c>
@@ -12588,7 +12592,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="176" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>56</v>
       </c>
@@ -12656,7 +12660,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="177" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>57</v>
       </c>
@@ -12724,7 +12728,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="178" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>58</v>
       </c>
@@ -12792,7 +12796,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="179" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>58</v>
       </c>
@@ -12860,7 +12864,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="180" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>58</v>
       </c>
@@ -12928,7 +12932,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="181" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>58</v>
       </c>
@@ -12996,7 +13000,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="182" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>58</v>
       </c>
@@ -13064,7 +13068,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="183" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>59</v>
       </c>
@@ -13132,7 +13136,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="184" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>59</v>
       </c>
@@ -13200,7 +13204,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="185" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>59</v>
       </c>
@@ -13268,7 +13272,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="186" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>59</v>
       </c>
@@ -13336,7 +13340,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="187" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>59</v>
       </c>
@@ -13404,7 +13408,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="188" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>59</v>
       </c>
@@ -13472,7 +13476,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="189" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>59</v>
       </c>
@@ -13540,7 +13544,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="190" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>59</v>
       </c>
@@ -13608,7 +13612,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="191" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>59</v>
       </c>
@@ -13676,7 +13680,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="192" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>59</v>
       </c>
@@ -13744,7 +13748,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="193" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>59</v>
       </c>
@@ -13812,7 +13816,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="194" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>59</v>
       </c>
@@ -13880,7 +13884,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="195" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>59</v>
       </c>
@@ -13948,7 +13952,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="196" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>59</v>
       </c>
@@ -14016,7 +14020,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="197" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>59</v>
       </c>
@@ -14084,7 +14088,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="198" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>59</v>
       </c>
@@ -14152,7 +14156,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="199" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>59</v>
       </c>
@@ -14220,7 +14224,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="200" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>60</v>
       </c>
@@ -14288,7 +14292,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="201" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>61</v>
       </c>
@@ -14356,7 +14360,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="202" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" t="s">
         <v>61</v>
       </c>
@@ -14424,7 +14428,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="203" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" t="s">
         <v>61</v>
       </c>
@@ -14492,7 +14496,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="204" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" t="s">
         <v>61</v>
       </c>
@@ -14560,7 +14564,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="205" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" t="s">
         <v>61</v>
       </c>
@@ -14628,7 +14632,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="206" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" t="s">
         <v>61</v>
       </c>
@@ -14696,7 +14700,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="207" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" t="s">
         <v>61</v>
       </c>
@@ -14764,7 +14768,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="208" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" t="s">
         <v>61</v>
       </c>
@@ -14832,7 +14836,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="209" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" t="s">
         <v>61</v>
       </c>
@@ -14900,7 +14904,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="210" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" t="s">
         <v>61</v>
       </c>
@@ -14968,7 +14972,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="211" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" t="s">
         <v>61</v>
       </c>
@@ -15036,7 +15040,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="212" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
         <v>61</v>
       </c>
@@ -15104,7 +15108,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="213" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
         <v>61</v>
       </c>
@@ -15172,7 +15176,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="214" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
         <v>61</v>
       </c>
@@ -15240,7 +15244,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="215" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
         <v>61</v>
       </c>
@@ -15308,7 +15312,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="216" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
         <v>62</v>
       </c>
@@ -15376,7 +15380,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="217" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
         <v>62</v>
       </c>
@@ -15444,7 +15448,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="218" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
         <v>62</v>
       </c>
@@ -15512,7 +15516,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="219" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
         <v>62</v>
       </c>
@@ -15580,7 +15584,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="220" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
         <v>62</v>
       </c>
@@ -15648,7 +15652,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="221" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
         <v>62</v>
       </c>
@@ -15716,7 +15720,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="222" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
         <v>62</v>
       </c>
@@ -15784,7 +15788,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="223" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
         <v>62</v>
       </c>
@@ -15852,7 +15856,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="224" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
         <v>62</v>
       </c>
@@ -15920,7 +15924,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="225" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
         <v>62</v>
       </c>
@@ -15988,7 +15992,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="226" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
         <v>62</v>
       </c>
@@ -16056,7 +16060,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="227" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
         <v>62</v>
       </c>
@@ -16124,7 +16128,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="228" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
         <v>62</v>
       </c>
@@ -16192,7 +16196,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="229" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
         <v>62</v>
       </c>
@@ -16260,7 +16264,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="230" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
         <v>62</v>
       </c>
@@ -16328,7 +16332,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="231" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
         <v>63</v>
       </c>
@@ -16396,7 +16400,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="232" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
         <v>63</v>
       </c>
@@ -16464,7 +16468,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="233" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
         <v>63</v>
       </c>
@@ -16532,7 +16536,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="234" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
         <v>63</v>
       </c>
@@ -16600,7 +16604,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="235" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
         <v>63</v>
       </c>
@@ -16668,7 +16672,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="236" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
         <v>63</v>
       </c>
@@ -16736,7 +16740,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="237" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
         <v>63</v>
       </c>
@@ -16804,7 +16808,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="238" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
         <v>63</v>
       </c>
@@ -16872,7 +16876,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="239" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" t="s">
         <v>63</v>
       </c>
@@ -16940,7 +16944,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="240" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" t="s">
         <v>64</v>
       </c>
@@ -17008,7 +17012,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="241" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" t="s">
         <v>64</v>
       </c>
@@ -17076,7 +17080,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="242" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" t="s">
         <v>64</v>
       </c>
@@ -17144,7 +17148,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="243" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" t="s">
         <v>64</v>
       </c>
@@ -17212,7 +17216,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="244" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" t="s">
         <v>64</v>
       </c>
@@ -17280,7 +17284,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="245" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" t="s">
         <v>64</v>
       </c>
@@ -17348,7 +17352,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="246" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" t="s">
         <v>64</v>
       </c>
@@ -17416,7 +17420,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="247" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" t="s">
         <v>64</v>
       </c>
@@ -17484,7 +17488,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="248" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" t="s">
         <v>64</v>
       </c>
@@ -17552,7 +17556,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="249" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" t="s">
         <v>64</v>
       </c>
@@ -17620,7 +17624,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="250" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" t="s">
         <v>64</v>
       </c>
@@ -17688,7 +17692,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="251" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" t="s">
         <v>64</v>
       </c>
@@ -17756,7 +17760,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="252" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" t="s">
         <v>64</v>
       </c>
@@ -17824,7 +17828,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="253" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" t="s">
         <v>65</v>
       </c>
@@ -17892,7 +17896,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="254" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
         <v>66</v>
       </c>
@@ -17960,7 +17964,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="255" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
         <v>66</v>
       </c>
@@ -18028,7 +18032,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="256" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
         <v>66</v>
       </c>
@@ -18096,7 +18100,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="257" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
         <v>66</v>
       </c>
@@ -18164,7 +18168,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="258" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" t="s">
         <v>66</v>
       </c>
@@ -18232,7 +18236,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="259" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" t="s">
         <v>66</v>
       </c>
@@ -18300,7 +18304,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="260" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" t="s">
         <v>67</v>
       </c>
@@ -18368,7 +18372,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="261" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" t="s">
         <v>67</v>
       </c>
@@ -18436,7 +18440,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="262" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A262" t="s">
         <v>67</v>
       </c>
@@ -18504,7 +18508,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="263" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" t="s">
         <v>67</v>
       </c>
@@ -18572,7 +18576,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="264" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>67</v>
       </c>
@@ -18640,7 +18644,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="265" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>67</v>
       </c>
@@ -18708,7 +18712,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="266" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>67</v>
       </c>
@@ -18776,7 +18780,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="267" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>67</v>
       </c>
@@ -18844,7 +18848,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="268" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" t="s">
         <v>67</v>
       </c>
@@ -18912,7 +18916,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="269" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>67</v>
       </c>
@@ -18980,7 +18984,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="270" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" t="s">
         <v>68</v>
       </c>
@@ -19048,7 +19052,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="271" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>68</v>
       </c>
@@ -19116,7 +19120,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="272" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>68</v>
       </c>
@@ -19184,7 +19188,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="273" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>68</v>
       </c>
@@ -19252,7 +19256,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="274" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>68</v>
       </c>
@@ -19320,7 +19324,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="275" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>68</v>
       </c>
@@ -19388,7 +19392,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="276" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>68</v>
       </c>
@@ -19456,7 +19460,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="277" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" t="s">
         <v>68</v>
       </c>
@@ -19524,7 +19528,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="278" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>68</v>
       </c>
@@ -19592,7 +19596,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="279" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" t="s">
         <v>68</v>
       </c>
@@ -19660,7 +19664,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="280" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:22" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" t="s">
         <v>68</v>
       </c>
@@ -19735,8 +19739,16 @@
       <c r="Q281" t="s">
         <v>88</v>
       </c>
+      <c r="V281">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="V1:V281" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="0">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>